<commit_message>
Added module-wise test cases
</commit_message>
<xml_diff>
--- a/Registration/regist.parabank.xlsx
+++ b/Registration/regist.parabank.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adars\Desktop\Manual Testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6DF32A2F-5549-4F5C-BE94-167F280570DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D34C0F5-9AAB-437B-92F8-F4AE0C47AA8B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{819CAF9A-015F-422C-9956-B8E34054A8AC}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="323" uniqueCount="194">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="324" uniqueCount="195">
   <si>
     <t>Test Case ID</t>
   </si>
@@ -525,6 +525,142 @@
   </si>
   <si>
     <t>cshcvsjhcg@gmail.com</t>
+  </si>
+  <si>
+    <t>Passwords did not match.Message displayed</t>
+  </si>
+  <si>
+    <t>Validation error displayed (“Password must be at least 6/8 characters”)</t>
+  </si>
+  <si>
+    <t>Validation message displayed (“Maximum length exceeded” or “Username should not exceed 20 characters”)</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Welcome 123
+"Your account was created successfully". You are now logged in </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>message displayed</t>
+    </r>
+  </si>
+  <si>
+    <t>Numeric in name (Invalid input validation)</t>
+  </si>
+  <si>
+    <t>Validation error displayed (“Name should contain only alphabets”)</t>
+  </si>
+  <si>
+    <t>Existing user "adarshs2506"</t>
+  </si>
+  <si>
+    <t>“This username already exists”</t>
+  </si>
+  <si>
+    <t>Open registration page → Check alignment, spacing, fields, buttons</t>
+  </si>
+  <si>
+    <t>All UI elements properly aligned and visible</t>
+  </si>
+  <si>
+    <t>"UI properly aligned"</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Cursor should move in correct navigation order
+(First Name → Last Name → Address → Username → Password → Submit)</t>
+  </si>
+  <si>
+    <t>"Cursor moves in correct sequence across all input fields".</t>
+  </si>
+  <si>
+    <t>…...</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+Data should be:
+Cleared OR
+Properly handled (no unintended submission / no stale data)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"Data not cleared after refresh"
+(Page retains previously entered data) </t>
+  </si>
+  <si>
+    <t>123– short/invalid number)</t>
+  </si>
+  <si>
+    <t>Validation error message displayed
+(“Please enter a valid phone number”)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+validation message: “Only alphabets allowed” Message displayed</t>
+  </si>
+  <si>
+    <t>56 chars</t>
+  </si>
+  <si>
+    <t>Leave all required fields blank → Click Submit</t>
+  </si>
+  <si>
+    <t>"Validation error" messages displayed for all mandatory fields</t>
+  </si>
+  <si>
+    <t>Error messages displayed for required fields (“First Name is required”
+“Last Name is required”
+“Username is required”
+“Password is required”etc)</t>
+  </si>
+  <si>
+    <t>"No validation error" message displayed</t>
+  </si>
+  <si>
+    <t>"Valid phone number accepted successfully", no validation error message displayed</t>
+  </si>
+  <si>
+    <t>1.Enter SQL query 
+2.Fill remaining fields with valid data 
+3. → Click Submit</t>
+  </si>
+  <si>
+    <t>Input should be blocked or validation message displayed. System should not allow unauthorized access or account creation</t>
+  </si>
+  <si>
+    <t>User is blocked with message “Sorry, you have been blocked / You are unable to access parasoft.com”</t>
+  </si>
+  <si>
+    <t>&lt;script&gt;alert('XSS')&lt;/script&gt;</t>
+  </si>
+  <si>
+    <t>Script should not execute or request should be blocked</t>
+  </si>
+  <si>
+    <t>Response should be fast (within 2–3 seconds)</t>
+  </si>
+  <si>
+    <t>Response received within "1 seconds"</t>
+  </si>
+  <si>
+    <t>Existing functionality should work properly</t>
+  </si>
+  <si>
+    <t>“Existing functionality works correctly as expected.”</t>
+  </si>
+  <si>
+    <t>"Registration works" successfully</t>
+  </si>
+  <si>
+    <t>Author:Adarsh Singh
+Reviewer:Projct Manager
+Approved by:Mr.Basab Roy
+Approval date:</t>
   </si>
   <si>
     <r>
@@ -553,7 +689,7 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t>"Your account was created successfully. You are now logged in".</t>
+      <t>"Your account was created successfully. You are now logged in".&amp; No validation error message displayed</t>
     </r>
     <r>
       <rPr>
@@ -564,18 +700,6 @@
       </rPr>
       <t xml:space="preserve"> </t>
     </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Message displayed</t>
-    </r>
-  </si>
-  <si>
-    <t>Passwords did not match.Message displayed</t>
   </si>
   <si>
     <r>
@@ -604,136 +728,8 @@
         <rFont val="Arial"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">"account was created successfully. You are now logged in".Message displayed
-</t>
+      <t>"account was created successfully. You are now logged in".Message displayed</t>
     </r>
-  </si>
-  <si>
-    <t>Validation error displayed (“Password must be at least 6/8 characters”)</t>
-  </si>
-  <si>
-    <t>Validation message displayed (“Maximum length exceeded” or “Username should not exceed 20 characters”)</t>
-  </si>
-  <si>
-    <r>
-      <t xml:space="preserve">Welcome 123
-"Your account was created successfully". You are now logged in </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>message displayed</t>
-    </r>
-  </si>
-  <si>
-    <t>Numeric in name (Invalid input validation)</t>
-  </si>
-  <si>
-    <t>Validation error displayed (“Name should contain only alphabets”)</t>
-  </si>
-  <si>
-    <t>Existing user "adarshs2506"</t>
-  </si>
-  <si>
-    <t>“This username already exists”</t>
-  </si>
-  <si>
-    <t>Open registration page → Check alignment, spacing, fields, buttons</t>
-  </si>
-  <si>
-    <t>All UI elements properly aligned and visible</t>
-  </si>
-  <si>
-    <t>"UI properly aligned"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Cursor should move in correct navigation order
-(First Name → Last Name → Address → Username → Password → Submit)</t>
-  </si>
-  <si>
-    <t>"Cursor moves in correct sequence across all input fields".</t>
-  </si>
-  <si>
-    <t>…...</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-Data should be:
-Cleared OR
-Properly handled (no unintended submission / no stale data)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">"Data not cleared after refresh"
-(Page retains previously entered data) </t>
-  </si>
-  <si>
-    <t>123– short/invalid number)</t>
-  </si>
-  <si>
-    <t>Validation error message displayed
-(“Please enter a valid phone number”)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-validation message: “Only alphabets allowed” Message displayed</t>
-  </si>
-  <si>
-    <t>56 chars</t>
-  </si>
-  <si>
-    <t>Leave all required fields blank → Click Submit</t>
-  </si>
-  <si>
-    <t>"Validation error" messages displayed for all mandatory fields</t>
-  </si>
-  <si>
-    <t>Error messages displayed for required fields (“First Name is required”
-“Last Name is required”
-“Username is required”
-“Password is required”etc)</t>
-  </si>
-  <si>
-    <t>"No validation error" message displayed</t>
-  </si>
-  <si>
-    <t>"Valid phone number accepted successfully", no validation error message displayed</t>
-  </si>
-  <si>
-    <t>1.Enter SQL query 
-2.Fill remaining fields with valid data 
-3. → Click Submit</t>
-  </si>
-  <si>
-    <t>Input should be blocked or validation message displayed. System should not allow unauthorized access or account creation</t>
-  </si>
-  <si>
-    <t>User is blocked with message “Sorry, you have been blocked / You are unable to access parasoft.com”</t>
-  </si>
-  <si>
-    <t>&lt;script&gt;alert('XSS')&lt;/script&gt;</t>
-  </si>
-  <si>
-    <t>Script should not execute or request should be blocked</t>
-  </si>
-  <si>
-    <t>Response should be fast (within 2–3 seconds)</t>
-  </si>
-  <si>
-    <t>Response received within "1 seconds"</t>
-  </si>
-  <si>
-    <t>Existing functionality should work properly</t>
-  </si>
-  <si>
-    <t>“Existing functionality works correctly as expected.”</t>
-  </si>
-  <si>
-    <t>"Registration works" successfully</t>
   </si>
 </sst>
 </file>
@@ -880,7 +876,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -914,22 +910,12 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -951,6 +937,19 @@
     <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1285,44 +1284,44 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E87967BC-3ECD-441C-92BE-D7065A18B1FE}">
-  <dimension ref="B3:U25"/>
+  <dimension ref="B3:U31"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="12.109375" customWidth="1"/>
     <col min="3" max="3" width="15" customWidth="1"/>
     <col min="4" max="4" width="35.33203125" customWidth="1"/>
-    <col min="5" max="5" width="23.44140625" style="18" customWidth="1"/>
+    <col min="5" max="5" width="23.44140625" customWidth="1"/>
     <col min="6" max="6" width="19.21875" customWidth="1"/>
     <col min="7" max="7" width="16.33203125" customWidth="1"/>
     <col min="8" max="8" width="23.5546875" customWidth="1"/>
-    <col min="9" max="9" width="21.33203125" style="16" customWidth="1"/>
+    <col min="9" max="9" width="26.109375" style="13" customWidth="1"/>
     <col min="10" max="10" width="8.21875" customWidth="1"/>
     <col min="11" max="11" width="10.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:21" ht="22.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="13" t="s">
+      <c r="B3" s="22" t="s">
         <v>69</v>
       </c>
-      <c r="C3" s="14"/>
-      <c r="D3" s="14"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14"/>
-      <c r="G3" s="14"/>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14"/>
-      <c r="T3" s="14"/>
-      <c r="U3" s="15"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="23"/>
+      <c r="F3" s="23"/>
+      <c r="G3" s="23"/>
+      <c r="H3" s="23"/>
+      <c r="I3" s="23"/>
+      <c r="J3" s="23"/>
+      <c r="K3" s="23"/>
+      <c r="L3" s="23"/>
+      <c r="M3" s="23"/>
+      <c r="N3" s="23"/>
+      <c r="O3" s="23"/>
+      <c r="P3" s="23"/>
+      <c r="Q3" s="23"/>
+      <c r="R3" s="23"/>
+      <c r="S3" s="23"/>
+      <c r="T3" s="23"/>
+      <c r="U3" s="24"/>
     </row>
     <row r="5" spans="2:21" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="5" t="s">
@@ -1334,7 +1333,7 @@
       <c r="D5" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="E5" s="17" t="s">
+      <c r="E5" s="14" t="s">
         <v>3</v>
       </c>
       <c r="F5" s="6" t="s">
@@ -1363,10 +1362,10 @@
       <c r="C6" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D6" s="20" t="s">
+      <c r="D6" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E6" s="23" t="s">
+      <c r="E6" s="19" t="s">
         <v>90</v>
       </c>
       <c r="F6" s="9" t="s">
@@ -1378,14 +1377,14 @@
       <c r="H6" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="I6" s="19" t="s">
+      <c r="I6" s="15" t="s">
         <v>154</v>
       </c>
-      <c r="J6" s="18" t="s">
+      <c r="J6" t="s">
         <v>71</v>
       </c>
       <c r="K6" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="7" spans="2:21" ht="103.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1395,11 +1394,11 @@
       <c r="C7" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D7" s="20" t="s">
+      <c r="D7" s="16" t="s">
         <v>150</v>
       </c>
       <c r="E7" s="9" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F7" s="9" t="s">
         <v>132</v>
@@ -1408,16 +1407,16 @@
         <v>94</v>
       </c>
       <c r="H7" s="9" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="I7" s="9" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="J7" s="9" t="s">
         <v>71</v>
       </c>
       <c r="K7" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="8" spans="2:21" ht="103.2" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
@@ -1427,30 +1426,31 @@
       <c r="C8" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D8" s="20" t="s">
+      <c r="D8" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E8" s="18" t="s">
+      <c r="E8" t="s">
         <v>96</v>
       </c>
       <c r="F8" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="G8" s="22" t="s">
+      <c r="G8" s="18" t="s">
         <v>156</v>
       </c>
       <c r="H8" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="I8" s="24" t="s">
-        <v>157</v>
+      <c r="I8" s="20" t="s">
+        <v>193</v>
       </c>
       <c r="J8" s="9" t="s">
         <v>155</v>
       </c>
       <c r="K8" s="9" t="s">
-        <v>172</v>
-      </c>
+        <v>170</v>
+      </c>
+      <c r="L8" s="26"/>
     </row>
     <row r="9" spans="2:21" ht="108" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B9" s="9" t="s">
@@ -1459,10 +1459,10 @@
       <c r="C9" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D9" s="20" t="s">
+      <c r="D9" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E9" s="18" t="s">
+      <c r="E9" t="s">
         <v>98</v>
       </c>
       <c r="F9" s="9" t="s">
@@ -1474,14 +1474,14 @@
       <c r="H9" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="I9" s="25" t="s">
-        <v>158</v>
+      <c r="I9" s="21" t="s">
+        <v>157</v>
       </c>
       <c r="J9" s="9" t="s">
         <v>71</v>
       </c>
       <c r="K9" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="10" spans="2:21" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1491,29 +1491,29 @@
       <c r="C10" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D10" s="20" t="s">
+      <c r="D10" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E10" s="18" t="s">
+      <c r="E10" t="s">
         <v>101</v>
       </c>
       <c r="F10" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="G10" s="23">
+      <c r="G10" s="19">
         <v>123</v>
       </c>
       <c r="H10" s="9" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="I10" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="J10" s="9" t="s">
         <v>155</v>
       </c>
       <c r="K10" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="11" spans="2:21" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1523,29 +1523,29 @@
       <c r="C11" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D11" s="20" t="s">
+      <c r="D11" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E11" s="18" t="s">
+      <c r="E11" t="s">
         <v>103</v>
       </c>
       <c r="F11" s="9" t="s">
         <v>138</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="H11" s="9" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="I11" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="J11" s="9" t="s">
         <v>155</v>
       </c>
       <c r="K11" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="12" spans="2:21" ht="105" customHeight="1" x14ac:dyDescent="0.3">
@@ -1555,10 +1555,10 @@
       <c r="C12" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D12" s="20" t="s">
+      <c r="D12" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E12" s="18" t="s">
+      <c r="E12" t="s">
         <v>105</v>
       </c>
       <c r="F12" s="9" t="s">
@@ -1568,16 +1568,16 @@
         <v>140</v>
       </c>
       <c r="H12" s="9" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="I12" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="J12" s="9" t="s">
         <v>155</v>
       </c>
       <c r="K12" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="13" spans="2:21" ht="100.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1587,29 +1587,29 @@
       <c r="C13" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D13" s="20" t="s">
+      <c r="D13" s="16" t="s">
         <v>150</v>
       </c>
       <c r="E13" s="9" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F13" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="G13" s="23">
+      <c r="G13" s="19">
         <v>123</v>
       </c>
       <c r="H13" s="9" t="s">
-        <v>164</v>
-      </c>
-      <c r="I13" s="22" t="s">
         <v>162</v>
+      </c>
+      <c r="I13" s="18" t="s">
+        <v>160</v>
       </c>
       <c r="J13" s="9" t="s">
         <v>155</v>
       </c>
       <c r="K13" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="14" spans="2:21" ht="103.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1619,29 +1619,29 @@
       <c r="C14" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D14" s="20" t="s">
+      <c r="D14" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E14" s="18" t="s">
+      <c r="E14" t="s">
         <v>108</v>
       </c>
       <c r="F14" s="9" t="s">
         <v>142</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="H14" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="I14" s="22" t="s">
-        <v>159</v>
+        <v>164</v>
+      </c>
+      <c r="I14" s="18" t="s">
+        <v>194</v>
       </c>
       <c r="J14" s="9" t="s">
         <v>155</v>
       </c>
       <c r="K14" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="15" spans="2:21" ht="105.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1651,29 +1651,29 @@
       <c r="C15" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D15" s="20" t="s">
+      <c r="D15" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E15" s="18" t="s">
+      <c r="E15" t="s">
         <v>110</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="G15" s="9" t="s">
         <v>48</v>
       </c>
       <c r="H15" s="9" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="I15" s="9" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="J15" s="9" t="s">
         <v>71</v>
       </c>
       <c r="K15" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="16" spans="2:21" ht="103.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1683,10 +1683,10 @@
       <c r="C16" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D16" s="20" t="s">
+      <c r="D16" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E16" s="18" t="s">
+      <c r="E16" t="s">
         <v>112</v>
       </c>
       <c r="F16" s="9" t="s">
@@ -1696,16 +1696,16 @@
         <v>48</v>
       </c>
       <c r="H16" s="9" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="I16" s="9" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="J16" s="9" t="s">
         <v>71</v>
       </c>
       <c r="K16" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="17" spans="2:11" ht="103.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1715,10 +1715,10 @@
       <c r="C17" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D17" s="20" t="s">
+      <c r="D17" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E17" s="18" t="s">
+      <c r="E17" t="s">
         <v>115</v>
       </c>
       <c r="F17" s="9" t="s">
@@ -1728,16 +1728,16 @@
         <v>48</v>
       </c>
       <c r="H17" s="9" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="I17" s="9" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="J17" s="9" t="s">
         <v>155</v>
       </c>
       <c r="K17" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="18" spans="2:11" ht="105" customHeight="1" x14ac:dyDescent="0.3">
@@ -1747,29 +1747,29 @@
       <c r="C18" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D18" s="20" t="s">
+      <c r="D18" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E18" s="18" t="s">
+      <c r="E18" t="s">
         <v>118</v>
       </c>
       <c r="F18" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="G18" s="23">
+      <c r="G18" s="19">
         <v>9876543210</v>
       </c>
       <c r="H18" s="9" t="s">
         <v>145</v>
       </c>
       <c r="I18" s="9" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="J18" s="9" t="s">
         <v>71</v>
       </c>
       <c r="K18" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="19" spans="2:11" ht="102.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1779,29 +1779,29 @@
       <c r="C19" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E19" s="18" t="s">
+      <c r="E19" t="s">
         <v>120</v>
       </c>
       <c r="F19" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="G19" s="23" t="s">
-        <v>175</v>
+      <c r="G19" s="19" t="s">
+        <v>173</v>
       </c>
       <c r="H19" s="9" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="I19" s="9" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="J19" s="9" t="s">
         <v>155</v>
       </c>
       <c r="K19" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="20" spans="2:11" ht="104.4" customHeight="1" x14ac:dyDescent="0.3">
@@ -1811,29 +1811,29 @@
       <c r="C20" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D20" s="20" t="s">
+      <c r="D20" s="16" t="s">
         <v>150</v>
       </c>
       <c r="E20" s="9" t="s">
         <v>122</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="G20" s="9" t="s">
         <v>123</v>
       </c>
       <c r="H20" s="9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="I20" s="9" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="J20" s="9" t="s">
         <v>71</v>
       </c>
       <c r="K20" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="21" spans="2:11" ht="103.8" customHeight="1" x14ac:dyDescent="0.3">
@@ -1843,29 +1843,29 @@
       <c r="C21" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D21" s="20" t="s">
+      <c r="D21" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E21" s="18" t="s">
+      <c r="E21" t="s">
         <v>125</v>
       </c>
       <c r="F21" s="9" t="s">
         <v>147</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="H21" s="9" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="I21" s="9" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="J21" s="9" t="s">
         <v>71</v>
       </c>
       <c r="K21" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="22" spans="2:11" ht="120.6" customHeight="1" x14ac:dyDescent="0.3">
@@ -1875,10 +1875,10 @@
       <c r="C22" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="20" t="s">
+      <c r="D22" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E22" s="18" t="s">
+      <c r="E22" t="s">
         <v>127</v>
       </c>
       <c r="F22" s="9" t="s">
@@ -1888,16 +1888,16 @@
         <v>129</v>
       </c>
       <c r="H22" s="9" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="I22" s="9" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="J22" s="9" t="s">
         <v>71</v>
       </c>
       <c r="K22" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="23" spans="2:11" ht="118.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -1907,10 +1907,10 @@
       <c r="C23" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D23" s="20" t="s">
+      <c r="D23" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E23" s="18" t="s">
+      <c r="E23" t="s">
         <v>148</v>
       </c>
       <c r="F23" s="9" t="s">
@@ -1920,32 +1920,32 @@
         <v>129</v>
       </c>
       <c r="H23" s="9" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="I23" s="9" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="J23" s="9" t="s">
         <v>71</v>
       </c>
       <c r="K23" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="24" spans="2:11" ht="100.8" x14ac:dyDescent="0.3">
-      <c r="B24" s="18" t="s">
+      <c r="B24" t="s">
         <v>130</v>
       </c>
       <c r="C24" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D24" s="20" t="s">
+      <c r="D24" s="16" t="s">
         <v>150</v>
       </c>
-      <c r="E24" s="18" t="s">
+      <c r="E24" t="s">
         <v>151</v>
       </c>
-      <c r="F24" s="18" t="s">
+      <c r="F24" t="s">
         <v>152</v>
       </c>
       <c r="G24" s="9" t="s">
@@ -1955,23 +1955,30 @@
         <v>153</v>
       </c>
       <c r="I24" s="9" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="J24" s="9" t="s">
         <v>71</v>
       </c>
       <c r="K24" s="9" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="25" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B25" s="18"/>
-      <c r="D25" s="21"/>
+      <c r="D25" s="17"/>
       <c r="I25" s="9"/>
     </row>
+    <row r="31" spans="2:11" ht="58.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="25" t="s">
+        <v>192</v>
+      </c>
+      <c r="C31" s="25"/>
+      <c r="D31" s="25"/>
+    </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="B3:U3"/>
+    <mergeCell ref="B31:D31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>